<commit_message>
Fix ECR column mapping for new PLI Online Apportionment column
The June ECR upload added a "PLI Online Apportionment" column (part of
the PLI/RPLI revenue component), shifting every column after it by one.
pipeline_config.yaml still pinned the old positions, so ECR validation
was failing silently and the dashboard was serving stale, understated
revenue/ECR figures for June. Shift the pinned columns, regenerate the
ECR upload template so BO Form submissions validate again, and rebuild
June's dataset with the corrected totals.
</commit_message>
<xml_diff>
--- a/templates/ecr.xlsx
+++ b/templates/ecr.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ECR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SWAP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECR" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SWAP" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK1"/>
+  <dimension ref="A1:AL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,40 +459,45 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>PLI Online Apportionment</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>Total PLI/RPLI Rev.</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Parcel</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>MO</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>IRGB</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>CCS</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Total revenue</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Exp. For ECR calculation</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>320107</t>
         </is>

</xml_diff>